<commit_message>
Remove the named authorization products
Owner direction, 20 October 2026: no references to the specific government and commercial
authorization systems the ATO Package Builder resembles. The builder now describes the work
the way authorization teams do it and calls itself an original practice tool, not an official
system of record. Course 2.1's text (materials edition 2.2, workbook rebuilt), the ATO Template
Library notes, the POA&M training sample, code comments, docs and AGENTS.md are reworded.
</commit_message>
<xml_diff>
--- a/public/training/library/training-samples/SBD-Training-POAM.xlsx
+++ b/public/training/library/training-samples/SBD-Training-POAM.xlsx
@@ -51,7 +51,7 @@
     <t xml:space="preserve">Columns</t>
   </si>
   <si>
-    <t xml:space="preserve">Field names follow CDSE's public POA&amp;M Job Aid (eMASS-style). One row per milestone: repeat the POA&amp;M ID on each milestone row of the same weakness.</t>
+    <t xml:space="preserve">Field names follow CDSE's public POA&amp;M Job Aid. One row per milestone: repeat the POA&amp;M ID on each milestone row of the same weakness.</t>
   </si>
   <si>
     <t xml:space="preserve">Risk</t>
@@ -87,7 +87,7 @@
     <t xml:space="preserve">Notice</t>
   </si>
   <si>
-    <t xml:space="preserve">Written by Secure By Design for training. Not the eMASS POA&amp;M or an official form.</t>
+    <t xml:space="preserve">Written by Secure By Design for training. Not an official form.</t>
   </si>
   <si>
     <t xml:space="preserve">Plan of Action and Milestones (POA&amp;M)</t>

</xml_diff>